<commit_message>
feat(arquivos_genericos):transformando arquivos em genericos
</commit_message>
<xml_diff>
--- a/Comparador_Console/Arquivos/ResultadoComparacao.xlsx
+++ b/Comparador_Console/Arquivos/ResultadoComparacao.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>ID</t>
   </si>
@@ -26,22 +26,40 @@
     <t>Valor B</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>GovernmentId</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>Cnpj</t>
+  </si>
+  <si>
+    <t>999</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
-    <t>GovernmentId</t>
-  </si>
-  <si>
     <t>456</t>
   </si>
   <si>
     <t>000</t>
   </si>
   <si>
+    <t>888</t>
+  </si>
+  <si>
     <t>3</t>
   </si>
   <si>
     <t>789</t>
+  </si>
+  <si>
+    <t>777</t>
   </si>
 </sst>
 </file>
@@ -87,7 +105,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr ">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -115,21 +133,77 @@
         <v>6</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="D3" s="0" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C4" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="B5" s="0" t="s">
         <v>7</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>